<commit_message>
Actualización automática de datos DGT (2026-08-05)
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-13T09:29:58+00:00</t>
+          <t>2026-08-05T08:30:43+00:00</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2015–2023 (9 años)</t>
+          <t>2015–2024 (10 años)</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4129,6 +4129,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4178,6 +4179,9 @@
       <c r="J4" s="7" t="n">
         <v>2023</v>
       </c>
+      <c r="K4" s="7" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -4212,6 +4216,9 @@
       <c r="J5" s="9" t="n">
         <v>717</v>
       </c>
+      <c r="K5" s="9" t="n">
+        <v>2152</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -4246,6 +4253,9 @@
       <c r="J6" s="9" t="n">
         <v>2244</v>
       </c>
+      <c r="K6" s="9" t="n">
+        <v>6337</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -4280,6 +4290,9 @@
       <c r="J7" s="9" t="n">
         <v>762</v>
       </c>
+      <c r="K7" s="9" t="n">
+        <v>2558</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -4314,6 +4327,9 @@
       <c r="J8" s="9" t="n">
         <v>0</v>
       </c>
+      <c r="K8" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -4348,6 +4364,9 @@
       <c r="J9" s="9" t="n">
         <v>528</v>
       </c>
+      <c r="K9" s="9" t="n">
+        <v>908</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -4382,6 +4401,9 @@
       <c r="J10" s="9" t="n">
         <v>348</v>
       </c>
+      <c r="K10" s="9" t="n">
+        <v>342</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -4416,6 +4438,9 @@
       <c r="J11" s="9" t="n">
         <v>28</v>
       </c>
+      <c r="K11" s="9" t="n">
+        <v>212</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -4450,6 +4475,9 @@
       <c r="J12" s="9" t="n">
         <v>42</v>
       </c>
+      <c r="K12" s="9" t="n">
+        <v>210</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -4484,6 +4512,9 @@
       <c r="J13" s="9" t="n">
         <v>54</v>
       </c>
+      <c r="K13" s="9" t="n">
+        <v>192</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -4518,6 +4549,9 @@
       <c r="J14" s="9" t="n">
         <v>6</v>
       </c>
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -4552,6 +4586,9 @@
       <c r="J15" s="9" t="n">
         <v>64</v>
       </c>
+      <c r="K15" s="9" t="n">
+        <v>364</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -4586,6 +4623,9 @@
       <c r="J16" s="9" t="n">
         <v>0</v>
       </c>
+      <c r="K16" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -4620,6 +4660,9 @@
       <c r="J17" s="9" t="n">
         <v>114</v>
       </c>
+      <c r="K17" s="9" t="n">
+        <v>291</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -4654,6 +4697,9 @@
       <c r="J18" s="9" t="n">
         <v>0</v>
       </c>
+      <c r="K18" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -4688,6 +4734,9 @@
       <c r="J19" s="9" t="n">
         <v>84</v>
       </c>
+      <c r="K19" s="9" t="n">
+        <v>402</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -4722,6 +4771,9 @@
       <c r="J20" s="9" t="n">
         <v>0</v>
       </c>
+      <c r="K20" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -4756,6 +4808,9 @@
       <c r="J21" s="9" t="n">
         <v>124</v>
       </c>
+      <c r="K21" s="9" t="n">
+        <v>416</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -4790,6 +4845,9 @@
       <c r="J22" s="9" t="n">
         <v>0</v>
       </c>
+      <c r="K22" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -4824,6 +4882,9 @@
       <c r="J23" s="9" t="n">
         <v>18</v>
       </c>
+      <c r="K23" s="9" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -4858,6 +4919,9 @@
       <c r="J24" s="9" t="n">
         <v>48</v>
       </c>
+      <c r="K24" s="9" t="n">
+        <v>232</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -4891,6 +4955,9 @@
       </c>
       <c r="J25" s="9" t="n">
         <v>24</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática de datos DGT (2026-10-05)
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-05T08:30:43+00:00</t>
+          <t>2026-10-05T13:33:05+00:00</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4467,7 @@
         <v>126</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="I12" s="9" t="n">
         <v>96</v>
@@ -4652,7 +4652,7 @@
         <v>498</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>894</v>
+        <v>849</v>
       </c>
       <c r="I17" s="9" t="n">
         <v>294</v>
@@ -4874,7 +4874,7 @@
         <v>99</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>48</v>
@@ -4948,7 +4948,7 @@
         <v>60</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="I25" s="9" t="n">
         <v>78</v>

</xml_diff>

<commit_message>
Datos DGT: sanciones y puntos 2024 (la Action estaba desactivada por inactividad)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Observatorio_Trafico_Marbella_DGT.xlsx
+++ b/Observatorio_Trafico_Marbella_DGT.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Aforos_MA341_MA417" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Criminalidad" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Comparativa_2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Indicadores" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Marbella" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Siniestralidad_Marbella" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sanciones_Marbella" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aforos_MA341_MA417" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criminalidad" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa_2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -557,7 +557,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-05T13:33:05+00:00</t>
+          <t>2026-10-27T13:34:05+00:00</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
         <v>7035003</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>38638981</v>
+        <v>38641163</v>
       </c>
     </row>
     <row r="8">
@@ -5701,7 +5701,7 @@
         <v>4488675</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>25786912</v>
+        <v>25788485</v>
       </c>
     </row>
     <row r="9">
@@ -5723,7 +5723,7 @@
         <v>896351</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>4510028</v>
+        <v>4510222</v>
       </c>
     </row>
     <row r="10">
@@ -5789,7 +5789,7 @@
         <v>281144</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>2341949</v>
+        <v>2341956</v>
       </c>
     </row>
     <row r="13">
@@ -5811,7 +5811,7 @@
         <v>1974555</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>9889957</v>
+        <v>9891048</v>
       </c>
     </row>
     <row r="14">

</xml_diff>